<commit_message>
Update: 1st to 10th
</commit_message>
<xml_diff>
--- a/data/steps.xlsx
+++ b/data/steps.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Date</t>
   </si>
@@ -54,6 +54,12 @@
   <si>
     <t>8-09-26</t>
   </si>
+  <si>
+    <t>9-09-26</t>
+  </si>
+  <si>
+    <t>10-09-26</t>
+  </si>
 </sst>
 </file>
 
@@ -86,12 +92,16 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -332,297 +342,862 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="3">
         <v>10623.0</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="3">
         <v>6000.0</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="3">
         <v>7611.0</v>
       </c>
-      <c r="E2" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="F2" s="2">
-        <v>1.0</v>
+      <c r="E2" s="3">
+        <v>7353.0</v>
+      </c>
+      <c r="F2" s="3">
+        <v>3816.0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="3">
         <v>11469.0</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="3">
         <v>3331.0</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="3">
         <v>15266.0</v>
       </c>
+      <c r="E3" s="3">
+        <v>4119.0</v>
+      </c>
+      <c r="F3" s="3">
+        <v>4206.0</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="3">
         <v>6003.0</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="3">
         <v>12568.0</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="3">
         <v>12625.0</v>
       </c>
+      <c r="E4" s="3">
+        <v>7469.0</v>
+      </c>
+      <c r="F4" s="3">
+        <v>3499.0</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="2">
-        <v>2084.0</v>
-      </c>
-      <c r="C5" s="2">
-        <v>8417.0</v>
-      </c>
-      <c r="D5" s="2">
-        <v>4924.0</v>
+      <c r="B5" s="3">
+        <v>7719.0</v>
+      </c>
+      <c r="C5" s="3">
+        <v>10503.0</v>
+      </c>
+      <c r="D5" s="3">
+        <v>10680.0</v>
+      </c>
+      <c r="E5" s="3">
+        <v>3043.0</v>
+      </c>
+      <c r="F5" s="3">
+        <v>2795.0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="B6" s="3">
+        <v>4084.0</v>
+      </c>
+      <c r="C6" s="3">
+        <v>1886.0</v>
+      </c>
+      <c r="D6" s="3">
+        <v>8499.0</v>
+      </c>
+      <c r="E6" s="3">
+        <v>7695.0</v>
+      </c>
+      <c r="F6" s="3">
+        <v>3055.0</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="B7" s="3">
+        <v>13263.0</v>
+      </c>
+      <c r="C7" s="3">
+        <v>11658.0</v>
+      </c>
+      <c r="D7" s="3">
+        <v>10320.0</v>
+      </c>
+      <c r="E7" s="3">
+        <v>11432.0</v>
+      </c>
+      <c r="F7" s="3">
+        <v>2931.0</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="B8" s="3">
+        <v>15637.0</v>
+      </c>
+      <c r="C8" s="3">
+        <v>10408.0</v>
+      </c>
+      <c r="D8" s="3">
+        <v>16601.0</v>
+      </c>
+      <c r="E8" s="3">
+        <v>7827.0</v>
+      </c>
+      <c r="F8" s="3">
+        <v>2617.0</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1"/>
-    <row r="22" ht="15.75" customHeight="1"/>
-    <row r="23" ht="15.75" customHeight="1"/>
-    <row r="24" ht="15.75" customHeight="1"/>
-    <row r="25" ht="15.75" customHeight="1"/>
-    <row r="26" ht="15.75" customHeight="1"/>
-    <row r="27" ht="15.75" customHeight="1"/>
-    <row r="28" ht="15.75" customHeight="1"/>
-    <row r="29" ht="15.75" customHeight="1"/>
-    <row r="30" ht="15.75" customHeight="1"/>
-    <row r="31" ht="15.75" customHeight="1"/>
-    <row r="32" ht="15.75" customHeight="1"/>
-    <row r="33" ht="15.75" customHeight="1"/>
-    <row r="34" ht="15.75" customHeight="1"/>
-    <row r="35" ht="15.75" customHeight="1"/>
-    <row r="36" ht="15.75" customHeight="1"/>
-    <row r="37" ht="15.75" customHeight="1"/>
-    <row r="38" ht="15.75" customHeight="1"/>
-    <row r="39" ht="15.75" customHeight="1"/>
-    <row r="40" ht="15.75" customHeight="1"/>
-    <row r="41" ht="15.75" customHeight="1"/>
-    <row r="42" ht="15.75" customHeight="1"/>
-    <row r="43" ht="15.75" customHeight="1"/>
-    <row r="44" ht="15.75" customHeight="1"/>
-    <row r="45" ht="15.75" customHeight="1"/>
-    <row r="46" ht="15.75" customHeight="1"/>
-    <row r="47" ht="15.75" customHeight="1"/>
-    <row r="48" ht="15.75" customHeight="1"/>
-    <row r="49" ht="15.75" customHeight="1"/>
-    <row r="50" ht="15.75" customHeight="1"/>
-    <row r="51" ht="15.75" customHeight="1"/>
-    <row r="52" ht="15.75" customHeight="1"/>
-    <row r="53" ht="15.75" customHeight="1"/>
-    <row r="54" ht="15.75" customHeight="1"/>
-    <row r="55" ht="15.75" customHeight="1"/>
-    <row r="56" ht="15.75" customHeight="1"/>
-    <row r="57" ht="15.75" customHeight="1"/>
-    <row r="58" ht="15.75" customHeight="1"/>
-    <row r="59" ht="15.75" customHeight="1"/>
-    <row r="60" ht="15.75" customHeight="1"/>
-    <row r="61" ht="15.75" customHeight="1"/>
-    <row r="62" ht="15.75" customHeight="1"/>
-    <row r="63" ht="15.75" customHeight="1"/>
-    <row r="64" ht="15.75" customHeight="1"/>
-    <row r="65" ht="15.75" customHeight="1"/>
-    <row r="66" ht="15.75" customHeight="1"/>
-    <row r="67" ht="15.75" customHeight="1"/>
-    <row r="68" ht="15.75" customHeight="1"/>
-    <row r="69" ht="15.75" customHeight="1"/>
-    <row r="70" ht="15.75" customHeight="1"/>
-    <row r="71" ht="15.75" customHeight="1"/>
-    <row r="72" ht="15.75" customHeight="1"/>
-    <row r="73" ht="15.75" customHeight="1"/>
-    <row r="74" ht="15.75" customHeight="1"/>
-    <row r="75" ht="15.75" customHeight="1"/>
-    <row r="76" ht="15.75" customHeight="1"/>
-    <row r="77" ht="15.75" customHeight="1"/>
-    <row r="78" ht="15.75" customHeight="1"/>
-    <row r="79" ht="15.75" customHeight="1"/>
-    <row r="80" ht="15.75" customHeight="1"/>
-    <row r="81" ht="15.75" customHeight="1"/>
-    <row r="82" ht="15.75" customHeight="1"/>
-    <row r="83" ht="15.75" customHeight="1"/>
-    <row r="84" ht="15.75" customHeight="1"/>
-    <row r="85" ht="15.75" customHeight="1"/>
-    <row r="86" ht="15.75" customHeight="1"/>
-    <row r="87" ht="15.75" customHeight="1"/>
-    <row r="88" ht="15.75" customHeight="1"/>
-    <row r="89" ht="15.75" customHeight="1"/>
-    <row r="90" ht="15.75" customHeight="1"/>
-    <row r="91" ht="15.75" customHeight="1"/>
-    <row r="92" ht="15.75" customHeight="1"/>
-    <row r="93" ht="15.75" customHeight="1"/>
-    <row r="94" ht="15.75" customHeight="1"/>
-    <row r="95" ht="15.75" customHeight="1"/>
-    <row r="96" ht="15.75" customHeight="1"/>
-    <row r="97" ht="15.75" customHeight="1"/>
-    <row r="98" ht="15.75" customHeight="1"/>
-    <row r="99" ht="15.75" customHeight="1"/>
-    <row r="100" ht="15.75" customHeight="1"/>
-    <row r="101" ht="15.75" customHeight="1"/>
-    <row r="102" ht="15.75" customHeight="1"/>
-    <row r="103" ht="15.75" customHeight="1"/>
-    <row r="104" ht="15.75" customHeight="1"/>
-    <row r="105" ht="15.75" customHeight="1"/>
-    <row r="106" ht="15.75" customHeight="1"/>
-    <row r="107" ht="15.75" customHeight="1"/>
-    <row r="108" ht="15.75" customHeight="1"/>
-    <row r="109" ht="15.75" customHeight="1"/>
-    <row r="110" ht="15.75" customHeight="1"/>
-    <row r="111" ht="15.75" customHeight="1"/>
-    <row r="112" ht="15.75" customHeight="1"/>
-    <row r="113" ht="15.75" customHeight="1"/>
-    <row r="114" ht="15.75" customHeight="1"/>
-    <row r="115" ht="15.75" customHeight="1"/>
-    <row r="116" ht="15.75" customHeight="1"/>
-    <row r="117" ht="15.75" customHeight="1"/>
-    <row r="118" ht="15.75" customHeight="1"/>
-    <row r="119" ht="15.75" customHeight="1"/>
-    <row r="120" ht="15.75" customHeight="1"/>
-    <row r="121" ht="15.75" customHeight="1"/>
-    <row r="122" ht="15.75" customHeight="1"/>
-    <row r="123" ht="15.75" customHeight="1"/>
-    <row r="124" ht="15.75" customHeight="1"/>
-    <row r="125" ht="15.75" customHeight="1"/>
-    <row r="126" ht="15.75" customHeight="1"/>
-    <row r="127" ht="15.75" customHeight="1"/>
-    <row r="128" ht="15.75" customHeight="1"/>
-    <row r="129" ht="15.75" customHeight="1"/>
-    <row r="130" ht="15.75" customHeight="1"/>
-    <row r="131" ht="15.75" customHeight="1"/>
-    <row r="132" ht="15.75" customHeight="1"/>
-    <row r="133" ht="15.75" customHeight="1"/>
-    <row r="134" ht="15.75" customHeight="1"/>
-    <row r="135" ht="15.75" customHeight="1"/>
-    <row r="136" ht="15.75" customHeight="1"/>
-    <row r="137" ht="15.75" customHeight="1"/>
-    <row r="138" ht="15.75" customHeight="1"/>
-    <row r="139" ht="15.75" customHeight="1"/>
-    <row r="140" ht="15.75" customHeight="1"/>
-    <row r="141" ht="15.75" customHeight="1"/>
-    <row r="142" ht="15.75" customHeight="1"/>
-    <row r="143" ht="15.75" customHeight="1"/>
-    <row r="144" ht="15.75" customHeight="1"/>
-    <row r="145" ht="15.75" customHeight="1"/>
-    <row r="146" ht="15.75" customHeight="1"/>
-    <row r="147" ht="15.75" customHeight="1"/>
-    <row r="148" ht="15.75" customHeight="1"/>
-    <row r="149" ht="15.75" customHeight="1"/>
-    <row r="150" ht="15.75" customHeight="1"/>
-    <row r="151" ht="15.75" customHeight="1"/>
-    <row r="152" ht="15.75" customHeight="1"/>
-    <row r="153" ht="15.75" customHeight="1"/>
-    <row r="154" ht="15.75" customHeight="1"/>
-    <row r="155" ht="15.75" customHeight="1"/>
-    <row r="156" ht="15.75" customHeight="1"/>
-    <row r="157" ht="15.75" customHeight="1"/>
-    <row r="158" ht="15.75" customHeight="1"/>
-    <row r="159" ht="15.75" customHeight="1"/>
-    <row r="160" ht="15.75" customHeight="1"/>
-    <row r="161" ht="15.75" customHeight="1"/>
-    <row r="162" ht="15.75" customHeight="1"/>
-    <row r="163" ht="15.75" customHeight="1"/>
-    <row r="164" ht="15.75" customHeight="1"/>
-    <row r="165" ht="15.75" customHeight="1"/>
-    <row r="166" ht="15.75" customHeight="1"/>
-    <row r="167" ht="15.75" customHeight="1"/>
-    <row r="168" ht="15.75" customHeight="1"/>
-    <row r="169" ht="15.75" customHeight="1"/>
-    <row r="170" ht="15.75" customHeight="1"/>
-    <row r="171" ht="15.75" customHeight="1"/>
-    <row r="172" ht="15.75" customHeight="1"/>
-    <row r="173" ht="15.75" customHeight="1"/>
-    <row r="174" ht="15.75" customHeight="1"/>
-    <row r="175" ht="15.75" customHeight="1"/>
-    <row r="176" ht="15.75" customHeight="1"/>
-    <row r="177" ht="15.75" customHeight="1"/>
-    <row r="178" ht="15.75" customHeight="1"/>
-    <row r="179" ht="15.75" customHeight="1"/>
-    <row r="180" ht="15.75" customHeight="1"/>
-    <row r="181" ht="15.75" customHeight="1"/>
-    <row r="182" ht="15.75" customHeight="1"/>
-    <row r="183" ht="15.75" customHeight="1"/>
-    <row r="184" ht="15.75" customHeight="1"/>
-    <row r="185" ht="15.75" customHeight="1"/>
-    <row r="186" ht="15.75" customHeight="1"/>
-    <row r="187" ht="15.75" customHeight="1"/>
-    <row r="188" ht="15.75" customHeight="1"/>
-    <row r="189" ht="15.75" customHeight="1"/>
-    <row r="190" ht="15.75" customHeight="1"/>
-    <row r="191" ht="15.75" customHeight="1"/>
-    <row r="192" ht="15.75" customHeight="1"/>
-    <row r="193" ht="15.75" customHeight="1"/>
-    <row r="194" ht="15.75" customHeight="1"/>
-    <row r="195" ht="15.75" customHeight="1"/>
-    <row r="196" ht="15.75" customHeight="1"/>
-    <row r="197" ht="15.75" customHeight="1"/>
-    <row r="198" ht="15.75" customHeight="1"/>
-    <row r="199" ht="15.75" customHeight="1"/>
-    <row r="200" ht="15.75" customHeight="1"/>
-    <row r="201" ht="15.75" customHeight="1"/>
-    <row r="202" ht="15.75" customHeight="1"/>
-    <row r="203" ht="15.75" customHeight="1"/>
-    <row r="204" ht="15.75" customHeight="1"/>
-    <row r="205" ht="15.75" customHeight="1"/>
-    <row r="206" ht="15.75" customHeight="1"/>
-    <row r="207" ht="15.75" customHeight="1"/>
-    <row r="208" ht="15.75" customHeight="1"/>
-    <row r="209" ht="15.75" customHeight="1"/>
-    <row r="210" ht="15.75" customHeight="1"/>
-    <row r="211" ht="15.75" customHeight="1"/>
-    <row r="212" ht="15.75" customHeight="1"/>
-    <row r="213" ht="15.75" customHeight="1"/>
-    <row r="214" ht="15.75" customHeight="1"/>
-    <row r="215" ht="15.75" customHeight="1"/>
-    <row r="216" ht="15.75" customHeight="1"/>
-    <row r="217" ht="15.75" customHeight="1"/>
-    <row r="218" ht="15.75" customHeight="1"/>
-    <row r="219" ht="15.75" customHeight="1"/>
-    <row r="220" ht="15.75" customHeight="1"/>
-    <row r="221" ht="15.75" customHeight="1"/>
-    <row r="222" ht="15.75" customHeight="1"/>
-    <row r="223" ht="15.75" customHeight="1"/>
-    <row r="224" ht="15.75" customHeight="1"/>
-    <row r="225" ht="15.75" customHeight="1"/>
-    <row r="226" ht="15.75" customHeight="1"/>
-    <row r="227" ht="15.75" customHeight="1"/>
-    <row r="228" ht="15.75" customHeight="1"/>
-    <row r="229" ht="15.75" customHeight="1"/>
-    <row r="230" ht="15.75" customHeight="1"/>
+      <c r="B9" s="3">
+        <v>10840.0</v>
+      </c>
+      <c r="C9" s="3">
+        <v>5634.0</v>
+      </c>
+      <c r="D9" s="3">
+        <v>11367.0</v>
+      </c>
+      <c r="E9" s="3">
+        <v>9217.0</v>
+      </c>
+      <c r="F9" s="3">
+        <v>4420.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="3">
+        <v>13739.0</v>
+      </c>
+      <c r="C10" s="3">
+        <v>10088.0</v>
+      </c>
+      <c r="D10" s="3">
+        <v>17597.0</v>
+      </c>
+      <c r="E10" s="3">
+        <v>6784.0</v>
+      </c>
+      <c r="F10" s="3">
+        <v>4854.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="3">
+        <v>1737.0</v>
+      </c>
+      <c r="C11" s="3">
+        <v>5566.0</v>
+      </c>
+      <c r="D11" s="3">
+        <v>11992.0</v>
+      </c>
+      <c r="E11" s="3">
+        <v>6251.0</v>
+      </c>
+      <c r="F11" s="3">
+        <v>3372.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2"/>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="2"/>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="2"/>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="2"/>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="2"/>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="2"/>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="2"/>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="2"/>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="2"/>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="2"/>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="2"/>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="2"/>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="2"/>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="2"/>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="2"/>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="2"/>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="2"/>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="2"/>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="2"/>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="2"/>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="A40" s="2"/>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="2"/>
+    </row>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="A42" s="2"/>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="A43" s="2"/>
+    </row>
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="A44" s="2"/>
+    </row>
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="A45" s="2"/>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="A46" s="2"/>
+    </row>
+    <row r="47" ht="15.75" customHeight="1">
+      <c r="A47" s="2"/>
+    </row>
+    <row r="48" ht="15.75" customHeight="1">
+      <c r="A48" s="2"/>
+    </row>
+    <row r="49" ht="15.75" customHeight="1">
+      <c r="A49" s="2"/>
+    </row>
+    <row r="50" ht="15.75" customHeight="1">
+      <c r="A50" s="2"/>
+    </row>
+    <row r="51" ht="15.75" customHeight="1">
+      <c r="A51" s="2"/>
+    </row>
+    <row r="52" ht="15.75" customHeight="1">
+      <c r="A52" s="2"/>
+    </row>
+    <row r="53" ht="15.75" customHeight="1">
+      <c r="A53" s="2"/>
+    </row>
+    <row r="54" ht="15.75" customHeight="1">
+      <c r="A54" s="2"/>
+    </row>
+    <row r="55" ht="15.75" customHeight="1">
+      <c r="A55" s="2"/>
+    </row>
+    <row r="56" ht="15.75" customHeight="1">
+      <c r="A56" s="2"/>
+    </row>
+    <row r="57" ht="15.75" customHeight="1">
+      <c r="A57" s="2"/>
+    </row>
+    <row r="58" ht="15.75" customHeight="1">
+      <c r="A58" s="2"/>
+    </row>
+    <row r="59" ht="15.75" customHeight="1">
+      <c r="A59" s="2"/>
+    </row>
+    <row r="60" ht="15.75" customHeight="1">
+      <c r="A60" s="2"/>
+    </row>
+    <row r="61" ht="15.75" customHeight="1">
+      <c r="A61" s="2"/>
+    </row>
+    <row r="62" ht="15.75" customHeight="1">
+      <c r="A62" s="2"/>
+    </row>
+    <row r="63" ht="15.75" customHeight="1">
+      <c r="A63" s="2"/>
+    </row>
+    <row r="64" ht="15.75" customHeight="1">
+      <c r="A64" s="2"/>
+    </row>
+    <row r="65" ht="15.75" customHeight="1">
+      <c r="A65" s="2"/>
+    </row>
+    <row r="66" ht="15.75" customHeight="1">
+      <c r="A66" s="2"/>
+    </row>
+    <row r="67" ht="15.75" customHeight="1">
+      <c r="A67" s="2"/>
+    </row>
+    <row r="68" ht="15.75" customHeight="1">
+      <c r="A68" s="2"/>
+    </row>
+    <row r="69" ht="15.75" customHeight="1">
+      <c r="A69" s="2"/>
+    </row>
+    <row r="70" ht="15.75" customHeight="1">
+      <c r="A70" s="2"/>
+    </row>
+    <row r="71" ht="15.75" customHeight="1">
+      <c r="A71" s="2"/>
+    </row>
+    <row r="72" ht="15.75" customHeight="1">
+      <c r="A72" s="2"/>
+    </row>
+    <row r="73" ht="15.75" customHeight="1">
+      <c r="A73" s="2"/>
+    </row>
+    <row r="74" ht="15.75" customHeight="1">
+      <c r="A74" s="2"/>
+    </row>
+    <row r="75" ht="15.75" customHeight="1">
+      <c r="A75" s="2"/>
+    </row>
+    <row r="76" ht="15.75" customHeight="1">
+      <c r="A76" s="2"/>
+    </row>
+    <row r="77" ht="15.75" customHeight="1">
+      <c r="A77" s="2"/>
+    </row>
+    <row r="78" ht="15.75" customHeight="1">
+      <c r="A78" s="2"/>
+    </row>
+    <row r="79" ht="15.75" customHeight="1">
+      <c r="A79" s="2"/>
+    </row>
+    <row r="80" ht="15.75" customHeight="1">
+      <c r="A80" s="2"/>
+    </row>
+    <row r="81" ht="15.75" customHeight="1">
+      <c r="A81" s="2"/>
+    </row>
+    <row r="82" ht="15.75" customHeight="1">
+      <c r="A82" s="2"/>
+    </row>
+    <row r="83" ht="15.75" customHeight="1">
+      <c r="A83" s="2"/>
+    </row>
+    <row r="84" ht="15.75" customHeight="1">
+      <c r="A84" s="2"/>
+    </row>
+    <row r="85" ht="15.75" customHeight="1">
+      <c r="A85" s="2"/>
+    </row>
+    <row r="86" ht="15.75" customHeight="1">
+      <c r="A86" s="2"/>
+    </row>
+    <row r="87" ht="15.75" customHeight="1">
+      <c r="A87" s="2"/>
+    </row>
+    <row r="88" ht="15.75" customHeight="1">
+      <c r="A88" s="2"/>
+    </row>
+    <row r="89" ht="15.75" customHeight="1">
+      <c r="A89" s="2"/>
+    </row>
+    <row r="90" ht="15.75" customHeight="1">
+      <c r="A90" s="2"/>
+    </row>
+    <row r="91" ht="15.75" customHeight="1">
+      <c r="A91" s="2"/>
+    </row>
+    <row r="92" ht="15.75" customHeight="1">
+      <c r="A92" s="2"/>
+    </row>
+    <row r="93" ht="15.75" customHeight="1">
+      <c r="A93" s="2"/>
+    </row>
+    <row r="94" ht="15.75" customHeight="1">
+      <c r="A94" s="2"/>
+    </row>
+    <row r="95" ht="15.75" customHeight="1">
+      <c r="A95" s="2"/>
+    </row>
+    <row r="96" ht="15.75" customHeight="1">
+      <c r="A96" s="2"/>
+    </row>
+    <row r="97" ht="15.75" customHeight="1">
+      <c r="A97" s="2"/>
+    </row>
+    <row r="98" ht="15.75" customHeight="1">
+      <c r="A98" s="2"/>
+    </row>
+    <row r="99" ht="15.75" customHeight="1">
+      <c r="A99" s="2"/>
+    </row>
+    <row r="100" ht="15.75" customHeight="1">
+      <c r="A100" s="2"/>
+    </row>
+    <row r="101" ht="15.75" customHeight="1">
+      <c r="A101" s="2"/>
+    </row>
+    <row r="102" ht="15.75" customHeight="1">
+      <c r="A102" s="2"/>
+    </row>
+    <row r="103" ht="15.75" customHeight="1">
+      <c r="A103" s="2"/>
+    </row>
+    <row r="104" ht="15.75" customHeight="1">
+      <c r="A104" s="2"/>
+    </row>
+    <row r="105" ht="15.75" customHeight="1">
+      <c r="A105" s="2"/>
+    </row>
+    <row r="106" ht="15.75" customHeight="1">
+      <c r="A106" s="2"/>
+    </row>
+    <row r="107" ht="15.75" customHeight="1">
+      <c r="A107" s="2"/>
+    </row>
+    <row r="108" ht="15.75" customHeight="1">
+      <c r="A108" s="2"/>
+    </row>
+    <row r="109" ht="15.75" customHeight="1">
+      <c r="A109" s="2"/>
+    </row>
+    <row r="110" ht="15.75" customHeight="1">
+      <c r="A110" s="2"/>
+    </row>
+    <row r="111" ht="15.75" customHeight="1">
+      <c r="A111" s="2"/>
+    </row>
+    <row r="112" ht="15.75" customHeight="1">
+      <c r="A112" s="2"/>
+    </row>
+    <row r="113" ht="15.75" customHeight="1">
+      <c r="A113" s="2"/>
+    </row>
+    <row r="114" ht="15.75" customHeight="1">
+      <c r="A114" s="2"/>
+    </row>
+    <row r="115" ht="15.75" customHeight="1">
+      <c r="A115" s="2"/>
+    </row>
+    <row r="116" ht="15.75" customHeight="1">
+      <c r="A116" s="2"/>
+    </row>
+    <row r="117" ht="15.75" customHeight="1">
+      <c r="A117" s="2"/>
+    </row>
+    <row r="118" ht="15.75" customHeight="1">
+      <c r="A118" s="2"/>
+    </row>
+    <row r="119" ht="15.75" customHeight="1">
+      <c r="A119" s="2"/>
+    </row>
+    <row r="120" ht="15.75" customHeight="1">
+      <c r="A120" s="2"/>
+    </row>
+    <row r="121" ht="15.75" customHeight="1">
+      <c r="A121" s="2"/>
+    </row>
+    <row r="122" ht="15.75" customHeight="1">
+      <c r="A122" s="2"/>
+    </row>
+    <row r="123" ht="15.75" customHeight="1">
+      <c r="A123" s="2"/>
+    </row>
+    <row r="124" ht="15.75" customHeight="1">
+      <c r="A124" s="2"/>
+    </row>
+    <row r="125" ht="15.75" customHeight="1">
+      <c r="A125" s="2"/>
+    </row>
+    <row r="126" ht="15.75" customHeight="1">
+      <c r="A126" s="2"/>
+    </row>
+    <row r="127" ht="15.75" customHeight="1">
+      <c r="A127" s="2"/>
+    </row>
+    <row r="128" ht="15.75" customHeight="1">
+      <c r="A128" s="2"/>
+    </row>
+    <row r="129" ht="15.75" customHeight="1">
+      <c r="A129" s="2"/>
+    </row>
+    <row r="130" ht="15.75" customHeight="1">
+      <c r="A130" s="2"/>
+    </row>
+    <row r="131" ht="15.75" customHeight="1">
+      <c r="A131" s="2"/>
+    </row>
+    <row r="132" ht="15.75" customHeight="1">
+      <c r="A132" s="2"/>
+    </row>
+    <row r="133" ht="15.75" customHeight="1">
+      <c r="A133" s="2"/>
+    </row>
+    <row r="134" ht="15.75" customHeight="1">
+      <c r="A134" s="2"/>
+    </row>
+    <row r="135" ht="15.75" customHeight="1">
+      <c r="A135" s="2"/>
+    </row>
+    <row r="136" ht="15.75" customHeight="1">
+      <c r="A136" s="2"/>
+    </row>
+    <row r="137" ht="15.75" customHeight="1">
+      <c r="A137" s="2"/>
+    </row>
+    <row r="138" ht="15.75" customHeight="1">
+      <c r="A138" s="2"/>
+    </row>
+    <row r="139" ht="15.75" customHeight="1">
+      <c r="A139" s="2"/>
+    </row>
+    <row r="140" ht="15.75" customHeight="1">
+      <c r="A140" s="2"/>
+    </row>
+    <row r="141" ht="15.75" customHeight="1">
+      <c r="A141" s="2"/>
+    </row>
+    <row r="142" ht="15.75" customHeight="1">
+      <c r="A142" s="2"/>
+    </row>
+    <row r="143" ht="15.75" customHeight="1">
+      <c r="A143" s="2"/>
+    </row>
+    <row r="144" ht="15.75" customHeight="1">
+      <c r="A144" s="2"/>
+    </row>
+    <row r="145" ht="15.75" customHeight="1">
+      <c r="A145" s="2"/>
+    </row>
+    <row r="146" ht="15.75" customHeight="1">
+      <c r="A146" s="2"/>
+    </row>
+    <row r="147" ht="15.75" customHeight="1">
+      <c r="A147" s="2"/>
+    </row>
+    <row r="148" ht="15.75" customHeight="1">
+      <c r="A148" s="2"/>
+    </row>
+    <row r="149" ht="15.75" customHeight="1">
+      <c r="A149" s="2"/>
+    </row>
+    <row r="150" ht="15.75" customHeight="1">
+      <c r="A150" s="2"/>
+    </row>
+    <row r="151" ht="15.75" customHeight="1">
+      <c r="A151" s="2"/>
+    </row>
+    <row r="152" ht="15.75" customHeight="1">
+      <c r="A152" s="2"/>
+    </row>
+    <row r="153" ht="15.75" customHeight="1">
+      <c r="A153" s="2"/>
+    </row>
+    <row r="154" ht="15.75" customHeight="1">
+      <c r="A154" s="2"/>
+    </row>
+    <row r="155" ht="15.75" customHeight="1">
+      <c r="A155" s="2"/>
+    </row>
+    <row r="156" ht="15.75" customHeight="1">
+      <c r="A156" s="2"/>
+    </row>
+    <row r="157" ht="15.75" customHeight="1">
+      <c r="A157" s="2"/>
+    </row>
+    <row r="158" ht="15.75" customHeight="1">
+      <c r="A158" s="2"/>
+    </row>
+    <row r="159" ht="15.75" customHeight="1">
+      <c r="A159" s="2"/>
+    </row>
+    <row r="160" ht="15.75" customHeight="1">
+      <c r="A160" s="2"/>
+    </row>
+    <row r="161" ht="15.75" customHeight="1">
+      <c r="A161" s="2"/>
+    </row>
+    <row r="162" ht="15.75" customHeight="1">
+      <c r="A162" s="2"/>
+    </row>
+    <row r="163" ht="15.75" customHeight="1">
+      <c r="A163" s="2"/>
+    </row>
+    <row r="164" ht="15.75" customHeight="1">
+      <c r="A164" s="2"/>
+    </row>
+    <row r="165" ht="15.75" customHeight="1">
+      <c r="A165" s="2"/>
+    </row>
+    <row r="166" ht="15.75" customHeight="1">
+      <c r="A166" s="2"/>
+    </row>
+    <row r="167" ht="15.75" customHeight="1">
+      <c r="A167" s="2"/>
+    </row>
+    <row r="168" ht="15.75" customHeight="1">
+      <c r="A168" s="2"/>
+    </row>
+    <row r="169" ht="15.75" customHeight="1">
+      <c r="A169" s="2"/>
+    </row>
+    <row r="170" ht="15.75" customHeight="1">
+      <c r="A170" s="2"/>
+    </row>
+    <row r="171" ht="15.75" customHeight="1">
+      <c r="A171" s="2"/>
+    </row>
+    <row r="172" ht="15.75" customHeight="1">
+      <c r="A172" s="2"/>
+    </row>
+    <row r="173" ht="15.75" customHeight="1">
+      <c r="A173" s="2"/>
+    </row>
+    <row r="174" ht="15.75" customHeight="1">
+      <c r="A174" s="2"/>
+    </row>
+    <row r="175" ht="15.75" customHeight="1">
+      <c r="A175" s="2"/>
+    </row>
+    <row r="176" ht="15.75" customHeight="1">
+      <c r="A176" s="2"/>
+    </row>
+    <row r="177" ht="15.75" customHeight="1">
+      <c r="A177" s="2"/>
+    </row>
+    <row r="178" ht="15.75" customHeight="1">
+      <c r="A178" s="2"/>
+    </row>
+    <row r="179" ht="15.75" customHeight="1">
+      <c r="A179" s="2"/>
+    </row>
+    <row r="180" ht="15.75" customHeight="1">
+      <c r="A180" s="2"/>
+    </row>
+    <row r="181" ht="15.75" customHeight="1">
+      <c r="A181" s="2"/>
+    </row>
+    <row r="182" ht="15.75" customHeight="1">
+      <c r="A182" s="2"/>
+    </row>
+    <row r="183" ht="15.75" customHeight="1">
+      <c r="A183" s="2"/>
+    </row>
+    <row r="184" ht="15.75" customHeight="1">
+      <c r="A184" s="2"/>
+    </row>
+    <row r="185" ht="15.75" customHeight="1">
+      <c r="A185" s="2"/>
+    </row>
+    <row r="186" ht="15.75" customHeight="1">
+      <c r="A186" s="2"/>
+    </row>
+    <row r="187" ht="15.75" customHeight="1">
+      <c r="A187" s="2"/>
+    </row>
+    <row r="188" ht="15.75" customHeight="1">
+      <c r="A188" s="2"/>
+    </row>
+    <row r="189" ht="15.75" customHeight="1">
+      <c r="A189" s="2"/>
+    </row>
+    <row r="190" ht="15.75" customHeight="1">
+      <c r="A190" s="2"/>
+    </row>
+    <row r="191" ht="15.75" customHeight="1">
+      <c r="A191" s="2"/>
+    </row>
+    <row r="192" ht="15.75" customHeight="1">
+      <c r="A192" s="2"/>
+    </row>
+    <row r="193" ht="15.75" customHeight="1">
+      <c r="A193" s="2"/>
+    </row>
+    <row r="194" ht="15.75" customHeight="1">
+      <c r="A194" s="2"/>
+    </row>
+    <row r="195" ht="15.75" customHeight="1">
+      <c r="A195" s="2"/>
+    </row>
+    <row r="196" ht="15.75" customHeight="1">
+      <c r="A196" s="2"/>
+    </row>
+    <row r="197" ht="15.75" customHeight="1">
+      <c r="A197" s="2"/>
+    </row>
+    <row r="198" ht="15.75" customHeight="1">
+      <c r="A198" s="2"/>
+    </row>
+    <row r="199" ht="15.75" customHeight="1">
+      <c r="A199" s="2"/>
+    </row>
+    <row r="200" ht="15.75" customHeight="1">
+      <c r="A200" s="2"/>
+    </row>
+    <row r="201" ht="15.75" customHeight="1">
+      <c r="A201" s="2"/>
+    </row>
+    <row r="202" ht="15.75" customHeight="1">
+      <c r="A202" s="2"/>
+    </row>
+    <row r="203" ht="15.75" customHeight="1">
+      <c r="A203" s="2"/>
+    </row>
+    <row r="204" ht="15.75" customHeight="1">
+      <c r="A204" s="2"/>
+    </row>
+    <row r="205" ht="15.75" customHeight="1">
+      <c r="A205" s="2"/>
+    </row>
+    <row r="206" ht="15.75" customHeight="1">
+      <c r="A206" s="2"/>
+    </row>
+    <row r="207" ht="15.75" customHeight="1">
+      <c r="A207" s="2"/>
+    </row>
+    <row r="208" ht="15.75" customHeight="1">
+      <c r="A208" s="2"/>
+    </row>
+    <row r="209" ht="15.75" customHeight="1">
+      <c r="A209" s="2"/>
+    </row>
+    <row r="210" ht="15.75" customHeight="1">
+      <c r="A210" s="2"/>
+    </row>
+    <row r="211" ht="15.75" customHeight="1">
+      <c r="A211" s="2"/>
+    </row>
+    <row r="212" ht="15.75" customHeight="1">
+      <c r="A212" s="2"/>
+    </row>
+    <row r="213" ht="15.75" customHeight="1">
+      <c r="A213" s="2"/>
+    </row>
+    <row r="214" ht="15.75" customHeight="1">
+      <c r="A214" s="2"/>
+    </row>
+    <row r="215" ht="15.75" customHeight="1">
+      <c r="A215" s="2"/>
+    </row>
+    <row r="216" ht="15.75" customHeight="1">
+      <c r="A216" s="2"/>
+    </row>
+    <row r="217" ht="15.75" customHeight="1">
+      <c r="A217" s="2"/>
+    </row>
+    <row r="218" ht="15.75" customHeight="1">
+      <c r="A218" s="2"/>
+    </row>
+    <row r="219" ht="15.75" customHeight="1">
+      <c r="A219" s="2"/>
+    </row>
+    <row r="220" ht="15.75" customHeight="1">
+      <c r="A220" s="2"/>
+    </row>
+    <row r="221" ht="15.75" customHeight="1">
+      <c r="A221" s="2"/>
+    </row>
+    <row r="222" ht="15.75" customHeight="1">
+      <c r="A222" s="2"/>
+    </row>
+    <row r="223" ht="15.75" customHeight="1">
+      <c r="A223" s="2"/>
+    </row>
+    <row r="224" ht="15.75" customHeight="1">
+      <c r="A224" s="2"/>
+    </row>
+    <row r="225" ht="15.75" customHeight="1">
+      <c r="A225" s="2"/>
+    </row>
+    <row r="226" ht="15.75" customHeight="1">
+      <c r="A226" s="2"/>
+    </row>
+    <row r="227" ht="15.75" customHeight="1">
+      <c r="A227" s="2"/>
+    </row>
+    <row r="228" ht="15.75" customHeight="1">
+      <c r="A228" s="2"/>
+    </row>
+    <row r="229" ht="15.75" customHeight="1">
+      <c r="A229" s="2"/>
+    </row>
+    <row r="230" ht="15.75" customHeight="1">
+      <c r="A230" s="2"/>
+    </row>
     <row r="231" ht="15.75" customHeight="1"/>
     <row r="232" ht="15.75" customHeight="1"/>
     <row r="233" ht="15.75" customHeight="1"/>

</xml_diff>